<commit_message>
StormGeo Data for the Production
</commit_message>
<xml_diff>
--- a/StormGeo Migration sheet for Go-Live.xlsx
+++ b/StormGeo Migration sheet for Go-Live.xlsx
@@ -5,22 +5,22 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pratiksha.bidgar\Desktop\StormGeo Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pratiksha.bidgar\Desktop\StormGeo Git\StormGeo_Personal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D69875-DC14-4F7D-AD6A-A80C3177726A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BE2CB3B-50B8-4C6D-8FE1-D6E7C00CEBC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Migration Sheet" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="126">
   <si>
     <t>Migration Fileds</t>
   </si>
@@ -49,9 +49,6 @@
     <t>Celigo Flows</t>
   </si>
   <si>
-    <t>Any hardcoded mapping</t>
-  </si>
-  <si>
     <t>Checklist</t>
   </si>
   <si>
@@ -88,15 +85,9 @@
     <t>SavedSearch</t>
   </si>
   <si>
-    <t>DF6: Salesforce Usage Place Holder to NetSuite Usage Flow</t>
-  </si>
-  <si>
     <t>Usage Place Holder Fields</t>
   </si>
   <si>
-    <t>Make_Usage_Void__c(Check Box)</t>
-  </si>
-  <si>
     <t>Order Product Fields</t>
   </si>
   <si>
@@ -121,9 +112,6 @@
     <t>Subscription Fields</t>
   </si>
   <si>
-    <t>NS_Subscription_Status__c(Free form text)</t>
-  </si>
-  <si>
     <t>[Celigo] Subscription Update</t>
   </si>
   <si>
@@ -136,12 +124,6 @@
     <t>Celigo Usage Search for subscription status ***Please don't delete***</t>
   </si>
   <si>
-    <t>DF 9: Product Status Updation from NS to SF</t>
-  </si>
-  <si>
-    <t>DF7:- Netsuite Usage Status Synch to Salesforce UPH</t>
-  </si>
-  <si>
     <t>SAT | Dummy Usage Record</t>
   </si>
   <si>
@@ -188,9 +170,6 @@
   </si>
   <si>
     <t>custrecordsf_subscription_status_updated</t>
-  </si>
-  <si>
-    <t>NetSuite Usage Status</t>
   </si>
   <si>
     <t>SF UPH Internal Id - is not empty</t>
@@ -355,17 +334,143 @@
   <si>
     <t>custrecord_vessel_sf_internal_id</t>
   </si>
+  <si>
+    <t>https://6812079-sb1.app.netsuite.com/app/common/scripting/script.nl?id=2444</t>
+  </si>
+  <si>
+    <t>SAT | SL | Usage Status Updation</t>
+  </si>
+  <si>
+    <t>Suitelet</t>
+  </si>
+  <si>
+    <t>SAT | Update status updation checkbox</t>
+  </si>
+  <si>
+    <t>UserEvent</t>
+  </si>
+  <si>
+    <t>https://6812079-sb1.app.netsuite.com/app/common/scripting/script.nl?id=2386</t>
+  </si>
+  <si>
+    <t>Subscription Change Order</t>
+  </si>
+  <si>
+    <t>SAT | UE | Custom Usage record creation</t>
+  </si>
+  <si>
+    <t>https://6812079-sb1.app.netsuite.com/app/common/scripting/script.nl?id=2442</t>
+  </si>
+  <si>
+    <t>Usage</t>
+  </si>
+  <si>
+    <t>Any hardcoded mapping/ NetSuite Scripts</t>
+  </si>
+  <si>
+    <t>custrecord_subscription_attached</t>
+  </si>
+  <si>
+    <t>Subscription Attached</t>
+  </si>
+  <si>
+    <t>Check all the Bundles</t>
+  </si>
+  <si>
+    <t>Not in use</t>
+  </si>
+  <si>
+    <t>Make_Usage_Void__c</t>
+  </si>
+  <si>
+    <t>Make Usage Void(Check Box)</t>
+  </si>
+  <si>
+    <t>NS Subscription Status(Free form text)</t>
+  </si>
+  <si>
+    <t>NS_Subscription_Status__c</t>
+  </si>
+  <si>
+    <t>Installed from the bundle - customscript_sbe_mu_voidrecords</t>
+  </si>
+  <si>
+    <t>UserEvent(Subscription Change Order)</t>
+  </si>
+  <si>
+    <t>UPH Updated(Check Box)</t>
+  </si>
+  <si>
+    <t>customsearch_celigo_subscription_update</t>
+  </si>
+  <si>
+    <t>customsearch_celigo_sat_usage_record_sta</t>
+  </si>
+  <si>
+    <t>customsearch_celigo_ops_subscription_sea</t>
+  </si>
+  <si>
+    <t>customsearch_celigo_sl_search</t>
+  </si>
+  <si>
+    <t>customscript_update_subscription_checkbo</t>
+  </si>
+  <si>
+    <t>customscript_sat_sl_usage_status_updatio</t>
+  </si>
+  <si>
+    <t>customscript_sat_usage_updated</t>
+  </si>
+  <si>
+    <t>NetSuite_Usage_Status__c</t>
+  </si>
+  <si>
+    <t>UPH_Updated__c</t>
+  </si>
+  <si>
+    <t>SAT | Usage void</t>
+  </si>
+  <si>
+    <t>DF 1: Product Status Updation from NS to SF</t>
+  </si>
+  <si>
+    <t>DF2: Salesforce Usage Place Holder to NetSuite Usage Flow</t>
+  </si>
+  <si>
+    <t>DF3:- Netsuite Usage Status Synch to Salesforce UPH</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -525,8 +630,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF262626"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF181818"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -566,6 +685,42 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF29B95C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF18B455"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F3F3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -642,18 +797,18 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -668,107 +823,203 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1074,7 +1325,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H168"/>
+  <dimension ref="A1:H179"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="27.6328125" bestFit="1" customWidth="1"/>
@@ -1114,15 +1365,15 @@
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="97" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2"/>
-      <c r="C2" s="24" t="s">
-        <v>22</v>
+      <c r="C2" s="101" t="s">
+        <v>124</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="2"/>
@@ -1130,13 +1381,13 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="42"/>
+      <c r="A3" s="98"/>
       <c r="B3" s="2"/>
-      <c r="C3" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="28" t="s">
-        <v>18</v>
+      <c r="C3" s="101" t="s">
+        <v>123</v>
+      </c>
+      <c r="D3" s="27" t="s">
+        <v>17</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="2"/>
@@ -1144,13 +1395,13 @@
       <c r="H3" s="2"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="42"/>
+      <c r="A4" s="98"/>
       <c r="B4" s="2"/>
-      <c r="C4" s="33" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>18</v>
+      <c r="C4" s="101" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>17</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="2"/>
@@ -1158,7 +1409,7 @@
       <c r="H4" s="2"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="42"/>
+      <c r="A5" s="98"/>
       <c r="B5" s="2"/>
       <c r="C5" s="7"/>
       <c r="D5" s="17"/>
@@ -1168,7 +1419,7 @@
       <c r="H5" s="2"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="42"/>
+      <c r="A6" s="98"/>
       <c r="B6" s="2"/>
       <c r="C6" s="16"/>
       <c r="D6" s="17"/>
@@ -1178,7 +1429,7 @@
       <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="42"/>
+      <c r="A7" s="98"/>
       <c r="B7" s="2"/>
       <c r="C7" s="15"/>
       <c r="D7" s="2"/>
@@ -1188,7 +1439,7 @@
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="42"/>
+      <c r="A8" s="98"/>
       <c r="B8" s="2"/>
       <c r="C8" s="7"/>
       <c r="D8" s="2"/>
@@ -1198,7 +1449,7 @@
       <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="42"/>
+      <c r="A9" s="98"/>
       <c r="B9" s="2"/>
       <c r="C9" s="7"/>
       <c r="D9" s="2"/>
@@ -1208,37 +1459,33 @@
       <c r="H9" s="2"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="42"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="42"/>
-      <c r="B11" s="2"/>
+      <c r="A10" s="98"/>
+      <c r="B10" s="44"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="44"/>
+    </row>
+    <row r="11" spans="1:8" s="2" customFormat="1">
+      <c r="A11" s="98"/>
       <c r="C11" s="7"/>
-      <c r="D11" s="2"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="2"/>
       <c r="G11" s="19"/>
-      <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="42"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="2"/>
+      <c r="A12" s="98"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="53"/>
+      <c r="H12" s="49"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="42"/>
+      <c r="A13" s="98"/>
       <c r="B13" s="2"/>
       <c r="C13" s="7"/>
       <c r="D13" s="2"/>
@@ -1248,7 +1495,7 @@
       <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="42"/>
+      <c r="A14" s="98"/>
       <c r="B14" s="2"/>
       <c r="C14" s="7"/>
       <c r="D14" s="2"/>
@@ -1258,7 +1505,7 @@
       <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="42"/>
+      <c r="A15" s="98"/>
       <c r="B15" s="2"/>
       <c r="C15" s="7"/>
       <c r="D15" s="2"/>
@@ -1267,8 +1514,8 @@
       <c r="G15" s="19"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" ht="13" customHeight="1">
-      <c r="A16" s="43"/>
+    <row r="16" spans="1:8">
+      <c r="A16" s="98"/>
       <c r="B16" s="2"/>
       <c r="C16" s="7"/>
       <c r="D16" s="2"/>
@@ -1277,34 +1524,32 @@
       <c r="G16" s="19"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="4"/>
+    <row r="17" spans="1:8" ht="13" customHeight="1">
+      <c r="A17" s="99"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="2"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="41" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="2"/>
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="4"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="42"/>
+      <c r="A19" s="97" t="s">
+        <v>18</v>
+      </c>
       <c r="B19" s="2"/>
-      <c r="C19" s="14" t="s">
-        <v>23</v>
-      </c>
+      <c r="C19" s="7"/>
       <c r="D19" s="2"/>
       <c r="E19" s="7"/>
       <c r="F19" s="2"/>
@@ -1312,127 +1557,127 @@
       <c r="H19" s="2"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="42"/>
+      <c r="A20" s="98"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="D20" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="C20" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" s="2"/>
       <c r="E20" s="7"/>
       <c r="F20" s="2"/>
       <c r="G20" s="19"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="42"/>
+      <c r="A21" s="98"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="27" t="s">
-        <v>91</v>
-      </c>
-      <c r="D21" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="27" t="s">
-        <v>56</v>
+      <c r="C21" s="89" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21" s="90" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="91"/>
+      <c r="F21" s="92" t="s">
+        <v>106</v>
       </c>
       <c r="G21" s="19"/>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="42"/>
+      <c r="A22" s="98"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="2"/>
+      <c r="C22" s="66" t="s">
+        <v>84</v>
+      </c>
+      <c r="D22" s="93" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="91"/>
+      <c r="F22" s="94" t="s">
+        <v>120</v>
+      </c>
       <c r="G22" s="19"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="42"/>
+      <c r="A23" s="98"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="19"/>
+      <c r="C23" s="66" t="s">
+        <v>112</v>
+      </c>
+      <c r="D23" s="95" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="91"/>
+      <c r="F23" s="96" t="s">
+        <v>121</v>
+      </c>
+      <c r="G23" s="88"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="42"/>
+      <c r="A24" s="98"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="25" t="s">
-        <v>20</v>
-      </c>
+      <c r="C24" s="73"/>
+      <c r="D24" s="29"/>
       <c r="E24" s="7"/>
-      <c r="F24" s="2"/>
+      <c r="F24" s="26"/>
       <c r="G24" s="19"/>
       <c r="H24" s="2"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="42"/>
+      <c r="A25" s="98"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="53"/>
-      <c r="D25" s="25"/>
+      <c r="C25" s="42"/>
+      <c r="D25" s="29"/>
       <c r="E25" s="7"/>
-      <c r="F25" s="2"/>
+      <c r="F25" s="26"/>
       <c r="G25" s="19"/>
       <c r="H25" s="2"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="42"/>
+      <c r="A26" s="98"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="51" t="s">
-        <v>54</v>
-      </c>
-      <c r="D26" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="7"/>
-      <c r="F26" s="27" t="s">
-        <v>55</v>
-      </c>
+      <c r="C26" s="24"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="2"/>
       <c r="G26" s="19"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="42"/>
+      <c r="A27" s="98"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="53" t="s">
-        <v>93</v>
-      </c>
-      <c r="D27" s="47" t="s">
-        <v>11</v>
-      </c>
+      <c r="C27" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27" s="2"/>
       <c r="E27" s="7"/>
-      <c r="F27" s="27" t="s">
-        <v>95</v>
-      </c>
+      <c r="F27" s="2"/>
       <c r="G27" s="19"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="42"/>
+      <c r="A28" s="98"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="2"/>
+      <c r="C28" s="102" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" s="103" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="91"/>
+      <c r="F28" s="92" t="s">
+        <v>109</v>
+      </c>
       <c r="G28" s="19"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="42"/>
+      <c r="A29" s="98"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="27"/>
+      <c r="C29" s="39"/>
       <c r="D29" s="25"/>
       <c r="E29" s="7"/>
       <c r="F29" s="2"/>
@@ -1440,149 +1685,159 @@
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="42"/>
+      <c r="A30" s="98"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="2"/>
+      <c r="C30" s="65" t="s">
+        <v>48</v>
+      </c>
+      <c r="D30" s="93" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="91"/>
+      <c r="F30" s="66" t="s">
+        <v>49</v>
+      </c>
       <c r="G30" s="19"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="42"/>
+      <c r="A31" s="98"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="52" t="s">
-        <v>32</v>
-      </c>
-      <c r="D31" s="25"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="2"/>
+      <c r="C31" s="66" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="104" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="91"/>
+      <c r="F31" s="102" t="s">
+        <v>88</v>
+      </c>
       <c r="G31" s="19"/>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="42"/>
+    <row r="32" spans="1:8" ht="15.5">
+      <c r="A32" s="98"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="53" t="s">
-        <v>53</v>
-      </c>
-      <c r="D32" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" s="7"/>
-      <c r="F32" s="2" t="s">
-        <v>52</v>
+      <c r="C32" s="64" t="s">
+        <v>103</v>
+      </c>
+      <c r="D32" s="105" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="91"/>
+      <c r="F32" s="106" t="s">
+        <v>102</v>
       </c>
       <c r="G32" s="19"/>
       <c r="H32" s="2"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="42"/>
+      <c r="A33" s="98"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="53" t="s">
-        <v>96</v>
-      </c>
-      <c r="D33" s="47" t="s">
-        <v>11</v>
-      </c>
+      <c r="C33" s="34"/>
+      <c r="D33" s="25"/>
       <c r="E33" s="7"/>
-      <c r="F33" s="27" t="s">
-        <v>97</v>
-      </c>
+      <c r="F33" s="2"/>
       <c r="G33" s="19"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="1:8">
-      <c r="A34" s="42"/>
+      <c r="A34" s="98"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="53"/>
-      <c r="D34" s="28"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="25"/>
       <c r="E34" s="7"/>
       <c r="F34" s="2"/>
       <c r="G34" s="19"/>
       <c r="H34" s="2"/>
     </row>
     <row r="35" spans="1:8">
-      <c r="A35" s="42"/>
+      <c r="A35" s="98"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="53"/>
-      <c r="D35" s="28"/>
+      <c r="C35" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="D35" s="25"/>
       <c r="E35" s="7"/>
       <c r="F35" s="2"/>
       <c r="G35" s="19"/>
       <c r="H35" s="2"/>
     </row>
     <row r="36" spans="1:8">
-      <c r="A36" s="42"/>
+      <c r="A36" s="98"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="53"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="2"/>
+      <c r="C36" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="D36" s="107" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" s="91"/>
+      <c r="F36" s="100" t="s">
+        <v>46</v>
+      </c>
       <c r="G36" s="19"/>
       <c r="H36" s="2"/>
     </row>
     <row r="37" spans="1:8">
-      <c r="A37" s="42"/>
+      <c r="A37" s="98"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="2"/>
+      <c r="C37" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37" s="104" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" s="91"/>
+      <c r="F37" s="102" t="s">
+        <v>90</v>
+      </c>
       <c r="G37" s="19"/>
       <c r="H37" s="2"/>
     </row>
     <row r="38" spans="1:8">
-      <c r="A38" s="42"/>
+      <c r="A38" s="98"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="25"/>
+      <c r="C38" s="39"/>
+      <c r="D38" s="27"/>
       <c r="E38" s="7"/>
       <c r="F38" s="2"/>
       <c r="G38" s="19"/>
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="1:8" ht="15" thickBot="1">
-      <c r="A39" s="42"/>
+    <row r="39" spans="1:8">
+      <c r="A39" s="98"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="D39" s="25"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="27"/>
       <c r="E39" s="7"/>
       <c r="F39" s="2"/>
       <c r="G39" s="19"/>
       <c r="H39" s="2"/>
     </row>
     <row r="40" spans="1:8">
-      <c r="A40" s="42"/>
+      <c r="A40" s="98"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="44" t="s">
-        <v>93</v>
-      </c>
-      <c r="D40" s="28" t="s">
-        <v>11</v>
-      </c>
+      <c r="C40" s="39"/>
+      <c r="D40" s="27"/>
       <c r="E40" s="7"/>
-      <c r="F40" s="46" t="s">
-        <v>94</v>
-      </c>
+      <c r="F40" s="2"/>
       <c r="G40" s="19"/>
       <c r="H40" s="2"/>
     </row>
     <row r="41" spans="1:8">
-      <c r="A41" s="42"/>
+      <c r="A41" s="98"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="25"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="27"/>
       <c r="E41" s="7"/>
-      <c r="F41" s="45"/>
+      <c r="F41" s="2"/>
       <c r="G41" s="19"/>
       <c r="H41" s="2"/>
     </row>
     <row r="42" spans="1:8">
-      <c r="A42" s="42"/>
+      <c r="A42" s="98"/>
       <c r="B42" s="2"/>
       <c r="C42" s="14"/>
       <c r="D42" s="25"/>
@@ -1591,10 +1846,12 @@
       <c r="G42" s="19"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="42"/>
+    <row r="43" spans="1:8" ht="15" thickBot="1">
+      <c r="A43" s="98"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="14"/>
+      <c r="C43" s="14" t="s">
+        <v>85</v>
+      </c>
       <c r="D43" s="25"/>
       <c r="E43" s="7"/>
       <c r="F43" s="2"/>
@@ -1602,849 +1859,857 @@
       <c r="H43" s="2"/>
     </row>
     <row r="44" spans="1:8">
-      <c r="A44" s="42"/>
+      <c r="A44" s="98"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="2"/>
+      <c r="C44" s="43" t="s">
+        <v>86</v>
+      </c>
+      <c r="D44" s="107" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="91"/>
+      <c r="F44" s="62" t="s">
+        <v>87</v>
+      </c>
       <c r="G44" s="19"/>
       <c r="H44" s="2"/>
     </row>
     <row r="45" spans="1:8">
-      <c r="A45" s="42"/>
+      <c r="A45" s="98"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="D45" s="17"/>
-      <c r="E45" s="16"/>
-      <c r="F45" s="2"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="25"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="34"/>
       <c r="G45" s="19"/>
       <c r="H45" s="2"/>
     </row>
     <row r="46" spans="1:8">
-      <c r="A46" s="42"/>
+      <c r="A46" s="98"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D46" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E46" s="16"/>
-      <c r="F46" s="27" t="s">
-        <v>49</v>
-      </c>
+      <c r="C46" s="14"/>
+      <c r="D46" s="25"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="2"/>
       <c r="G46" s="19"/>
       <c r="H46" s="2"/>
     </row>
     <row r="47" spans="1:8">
-      <c r="A47" s="42"/>
+      <c r="A47" s="98"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="D47" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E47" s="16"/>
-      <c r="F47" s="27" t="s">
-        <v>50</v>
-      </c>
+      <c r="C47" s="14"/>
+      <c r="D47" s="25"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="2"/>
       <c r="G47" s="19"/>
       <c r="H47" s="2"/>
     </row>
     <row r="48" spans="1:8">
-      <c r="A48" s="42"/>
+      <c r="A48" s="98"/>
       <c r="B48" s="2"/>
-      <c r="C48" s="48"/>
-      <c r="D48" s="12"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="2"/>
       <c r="E48" s="7"/>
-      <c r="F48" s="12"/>
+      <c r="F48" s="2"/>
       <c r="G48" s="19"/>
       <c r="H48" s="2"/>
     </row>
     <row r="49" spans="1:8">
-      <c r="A49" s="42"/>
+      <c r="A49" s="98"/>
       <c r="B49" s="2"/>
-      <c r="C49" s="50" t="s">
-        <v>40</v>
-      </c>
-      <c r="D49" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E49" s="7"/>
-      <c r="F49" s="12"/>
+      <c r="C49" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D49" s="17"/>
+      <c r="E49" s="16"/>
+      <c r="F49" s="2"/>
       <c r="G49" s="19"/>
       <c r="H49" s="2"/>
     </row>
     <row r="50" spans="1:8">
-      <c r="A50" s="42"/>
+      <c r="A50" s="98"/>
       <c r="B50" s="2"/>
-      <c r="C50" s="51" t="s">
-        <v>42</v>
-      </c>
-      <c r="D50" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" s="7"/>
-      <c r="F50" s="27" t="s">
-        <v>41</v>
+      <c r="C50" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="D50" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" s="16"/>
+      <c r="F50" s="26" t="s">
+        <v>43</v>
       </c>
       <c r="G50" s="19"/>
       <c r="H50" s="2"/>
     </row>
     <row r="51" spans="1:8">
-      <c r="A51" s="42"/>
+      <c r="A51" s="98"/>
       <c r="B51" s="2"/>
-      <c r="C51" s="51" t="s">
-        <v>43</v>
-      </c>
-      <c r="D51" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E51" s="7"/>
-      <c r="F51" s="27" t="s">
-        <v>46</v>
+      <c r="C51" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="D51" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" s="16"/>
+      <c r="F51" s="26" t="s">
+        <v>44</v>
       </c>
       <c r="G51" s="19"/>
       <c r="H51" s="2"/>
     </row>
     <row r="52" spans="1:8">
-      <c r="A52" s="42"/>
+      <c r="A52" s="98"/>
       <c r="B52" s="2"/>
-      <c r="C52" s="51" t="s">
-        <v>44</v>
-      </c>
-      <c r="D52" s="34" t="s">
-        <v>11</v>
-      </c>
+      <c r="C52" s="35"/>
+      <c r="D52" s="12"/>
       <c r="E52" s="7"/>
-      <c r="F52" s="27" t="s">
-        <v>47</v>
-      </c>
+      <c r="F52" s="12"/>
       <c r="G52" s="19"/>
       <c r="H52" s="2"/>
     </row>
     <row r="53" spans="1:8">
-      <c r="A53" s="42"/>
+      <c r="A53" s="98"/>
       <c r="B53" s="2"/>
-      <c r="C53" s="51" t="s">
-        <v>45</v>
-      </c>
-      <c r="D53" s="34" t="s">
-        <v>11</v>
+      <c r="C53" s="56" t="s">
+        <v>34</v>
+      </c>
+      <c r="D53" s="29" t="s">
+        <v>10</v>
       </c>
       <c r="E53" s="7"/>
-      <c r="F53" s="27" t="s">
-        <v>48</v>
-      </c>
+      <c r="F53" s="12"/>
       <c r="G53" s="19"/>
       <c r="H53" s="2"/>
     </row>
     <row r="54" spans="1:8">
-      <c r="A54" s="42"/>
+      <c r="A54" s="98"/>
       <c r="B54" s="2"/>
-      <c r="C54" s="49"/>
-      <c r="D54" s="12"/>
+      <c r="C54" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="D54" s="29" t="s">
+        <v>10</v>
+      </c>
       <c r="E54" s="7"/>
-      <c r="F54" s="12"/>
+      <c r="F54" s="26" t="s">
+        <v>35</v>
+      </c>
       <c r="G54" s="19"/>
       <c r="H54" s="2"/>
     </row>
     <row r="55" spans="1:8">
-      <c r="A55" s="42"/>
+      <c r="A55" s="98"/>
       <c r="B55" s="2"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="12"/>
+      <c r="C55" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="D55" s="29" t="s">
+        <v>10</v>
+      </c>
       <c r="E55" s="7"/>
-      <c r="F55" s="12"/>
+      <c r="F55" s="26" t="s">
+        <v>40</v>
+      </c>
       <c r="G55" s="19"/>
       <c r="H55" s="2"/>
     </row>
     <row r="56" spans="1:8">
-      <c r="A56" s="42"/>
+      <c r="A56" s="98"/>
       <c r="B56" s="2"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="12"/>
+      <c r="C56" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="D56" s="29" t="s">
+        <v>10</v>
+      </c>
       <c r="E56" s="7"/>
-      <c r="F56" s="12"/>
+      <c r="F56" s="26" t="s">
+        <v>41</v>
+      </c>
       <c r="G56" s="19"/>
       <c r="H56" s="2"/>
     </row>
     <row r="57" spans="1:8">
-      <c r="A57" s="42"/>
+      <c r="A57" s="98"/>
       <c r="B57" s="2"/>
-      <c r="C57" s="14"/>
-      <c r="D57" s="2"/>
+      <c r="C57" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="D57" s="29" t="s">
+        <v>10</v>
+      </c>
       <c r="E57" s="7"/>
-      <c r="F57" s="2"/>
+      <c r="F57" s="26" t="s">
+        <v>42</v>
+      </c>
       <c r="G57" s="19"/>
       <c r="H57" s="2"/>
     </row>
     <row r="58" spans="1:8">
-      <c r="A58" s="43"/>
+      <c r="A58" s="98"/>
       <c r="B58" s="2"/>
-      <c r="C58" s="7"/>
-      <c r="D58" s="2"/>
+      <c r="C58" s="36"/>
+      <c r="D58" s="12"/>
       <c r="E58" s="7"/>
-      <c r="F58" s="2"/>
+      <c r="F58" s="12"/>
       <c r="G58" s="19"/>
       <c r="H58" s="2"/>
     </row>
     <row r="59" spans="1:8">
-      <c r="A59" s="3"/>
-      <c r="B59" s="5"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="5"/>
-      <c r="G59" s="21"/>
-      <c r="H59" s="5"/>
+      <c r="A59" s="98"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="19"/>
+      <c r="H59" s="2"/>
     </row>
     <row r="60" spans="1:8">
-      <c r="A60" s="42" t="s">
-        <v>21</v>
-      </c>
+      <c r="A60" s="98"/>
       <c r="B60" s="2"/>
-      <c r="C60" s="16"/>
-      <c r="D60" s="13"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="12"/>
       <c r="E60" s="7"/>
-      <c r="F60" s="2"/>
+      <c r="F60" s="12"/>
       <c r="G60" s="19"/>
       <c r="H60" s="2"/>
     </row>
     <row r="61" spans="1:8">
-      <c r="A61" s="42"/>
+      <c r="A61" s="98"/>
       <c r="B61" s="2"/>
-      <c r="C61" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="D61" s="13"/>
+      <c r="C61" s="14"/>
+      <c r="D61" s="2"/>
       <c r="E61" s="7"/>
       <c r="F61" s="2"/>
       <c r="G61" s="19"/>
       <c r="H61" s="2"/>
     </row>
     <row r="62" spans="1:8">
-      <c r="A62" s="42"/>
+      <c r="A62" s="99"/>
       <c r="B62" s="2"/>
-      <c r="C62" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="D62" s="13" t="s">
-        <v>11</v>
-      </c>
+      <c r="C62" s="7"/>
+      <c r="D62" s="2"/>
       <c r="E62" s="7"/>
       <c r="F62" s="2"/>
       <c r="G62" s="19"/>
       <c r="H62" s="2"/>
     </row>
     <row r="63" spans="1:8">
-      <c r="A63" s="42"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="D63" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E63" s="7"/>
-      <c r="F63" s="2"/>
-      <c r="G63" s="19"/>
-      <c r="H63" s="2"/>
+      <c r="A63" s="3"/>
+      <c r="B63" s="5"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="9"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="21"/>
+      <c r="H63" s="5"/>
     </row>
     <row r="64" spans="1:8">
-      <c r="A64" s="42"/>
+      <c r="A64" s="98" t="s">
+        <v>20</v>
+      </c>
       <c r="B64" s="2"/>
-      <c r="C64" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="D64" s="31" t="s">
-        <v>11</v>
-      </c>
+      <c r="C64" s="16"/>
+      <c r="D64" s="13"/>
       <c r="E64" s="7"/>
       <c r="F64" s="2"/>
       <c r="G64" s="19"/>
       <c r="H64" s="2"/>
     </row>
     <row r="65" spans="1:8">
-      <c r="A65" s="42"/>
+      <c r="A65" s="98"/>
       <c r="B65" s="2"/>
-      <c r="C65" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="D65" s="28" t="s">
-        <v>36</v>
-      </c>
+      <c r="C65" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D65" s="13"/>
       <c r="E65" s="7"/>
       <c r="F65" s="2"/>
       <c r="G65" s="19"/>
       <c r="H65" s="2"/>
     </row>
     <row r="66" spans="1:8">
-      <c r="A66" s="42"/>
+      <c r="A66" s="98"/>
       <c r="B66" s="2"/>
-      <c r="C66" s="24"/>
-      <c r="D66" s="28"/>
+      <c r="C66" s="76" t="s">
+        <v>26</v>
+      </c>
+      <c r="D66" s="13" t="s">
+        <v>10</v>
+      </c>
       <c r="E66" s="7"/>
-      <c r="F66" s="2"/>
+      <c r="F66" s="77" t="s">
+        <v>115</v>
+      </c>
       <c r="G66" s="19"/>
       <c r="H66" s="2"/>
     </row>
     <row r="67" spans="1:8">
-      <c r="A67" s="42"/>
+      <c r="A67" s="98"/>
       <c r="B67" s="2"/>
-      <c r="C67" s="24"/>
-      <c r="D67" s="28"/>
+      <c r="C67" s="68" t="s">
+        <v>27</v>
+      </c>
+      <c r="D67" s="13" t="s">
+        <v>10</v>
+      </c>
       <c r="E67" s="7"/>
-      <c r="F67" s="2"/>
+      <c r="F67" s="87" t="s">
+        <v>116</v>
+      </c>
       <c r="G67" s="19"/>
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="1:8">
-      <c r="A68" s="42"/>
-      <c r="B68" s="2">
-        <v>1</v>
-      </c>
-      <c r="C68" s="39" t="s">
-        <v>29</v>
-      </c>
-      <c r="D68" s="28"/>
-      <c r="E68" s="7"/>
-      <c r="F68" s="2"/>
-      <c r="G68" s="19"/>
-      <c r="H68" s="2"/>
+    <row r="68" spans="1:8" s="83" customFormat="1">
+      <c r="A68" s="98"/>
+      <c r="B68" s="69" t="s">
+        <v>105</v>
+      </c>
+      <c r="C68" s="78" t="s">
+        <v>33</v>
+      </c>
+      <c r="D68" s="79" t="s">
+        <v>10</v>
+      </c>
+      <c r="E68" s="80"/>
+      <c r="F68" s="81"/>
+      <c r="G68" s="82"/>
+      <c r="H68" s="81"/>
     </row>
     <row r="69" spans="1:8">
-      <c r="A69" s="42"/>
+      <c r="A69" s="98"/>
       <c r="B69" s="2"/>
-      <c r="C69" s="33" t="s">
-        <v>72</v>
-      </c>
-      <c r="D69" s="28"/>
+      <c r="C69" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D69" s="27" t="s">
+        <v>32</v>
+      </c>
       <c r="E69" s="7"/>
       <c r="F69" s="2"/>
       <c r="G69" s="19"/>
       <c r="H69" s="2"/>
     </row>
     <row r="70" spans="1:8">
-      <c r="A70" s="42"/>
+      <c r="A70" s="98"/>
       <c r="B70" s="2"/>
-      <c r="C70" s="33" t="s">
-        <v>73</v>
-      </c>
-      <c r="D70" s="28"/>
+      <c r="C70" s="24"/>
+      <c r="D70" s="27"/>
       <c r="E70" s="7"/>
       <c r="F70" s="2"/>
       <c r="G70" s="19"/>
       <c r="H70" s="2"/>
     </row>
     <row r="71" spans="1:8">
-      <c r="A71" s="42"/>
+      <c r="A71" s="98"/>
       <c r="B71" s="2"/>
-      <c r="C71" s="33" t="s">
-        <v>74</v>
-      </c>
-      <c r="D71" s="28"/>
+      <c r="C71" s="24"/>
+      <c r="D71" s="27"/>
       <c r="E71" s="7"/>
       <c r="F71" s="2"/>
       <c r="G71" s="19"/>
       <c r="H71" s="2"/>
     </row>
     <row r="72" spans="1:8">
-      <c r="A72" s="42"/>
-      <c r="B72" s="2"/>
-      <c r="C72" s="24"/>
-      <c r="D72" s="28"/>
+      <c r="A72" s="98"/>
+      <c r="B72" s="2">
+        <v>1</v>
+      </c>
+      <c r="C72" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D72" s="2"/>
       <c r="E72" s="7"/>
       <c r="F72" s="2"/>
       <c r="G72" s="19"/>
       <c r="H72" s="2"/>
     </row>
     <row r="73" spans="1:8">
-      <c r="A73" s="42"/>
-      <c r="B73" s="2">
-        <v>2</v>
-      </c>
-      <c r="C73" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D73" s="28"/>
+      <c r="A73" s="98"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="D73" s="27"/>
       <c r="E73" s="7"/>
       <c r="F73" s="2"/>
       <c r="G73" s="19"/>
       <c r="H73" s="2"/>
     </row>
     <row r="74" spans="1:8">
-      <c r="A74" s="42"/>
+      <c r="A74" s="98"/>
       <c r="B74" s="2"/>
-      <c r="C74" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="D74" s="28"/>
+      <c r="C74" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="D74" s="27"/>
       <c r="E74" s="7"/>
       <c r="F74" s="2"/>
       <c r="G74" s="19"/>
       <c r="H74" s="2"/>
     </row>
     <row r="75" spans="1:8">
-      <c r="A75" s="42"/>
+      <c r="A75" s="98"/>
       <c r="B75" s="2"/>
-      <c r="C75" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="D75" s="28"/>
+      <c r="C75" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D75" s="27"/>
       <c r="E75" s="7"/>
       <c r="F75" s="2"/>
       <c r="G75" s="19"/>
       <c r="H75" s="2"/>
     </row>
     <row r="76" spans="1:8">
-      <c r="A76" s="42"/>
+      <c r="A76" s="98"/>
       <c r="B76" s="2"/>
-      <c r="C76" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D76" s="28"/>
+      <c r="C76" s="24"/>
+      <c r="D76" s="27"/>
       <c r="E76" s="7"/>
       <c r="F76" s="2"/>
       <c r="G76" s="19"/>
       <c r="H76" s="2"/>
     </row>
     <row r="77" spans="1:8">
-      <c r="A77" s="42"/>
-      <c r="B77" s="2"/>
-      <c r="C77" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="D77" s="28"/>
+      <c r="A77" s="98"/>
+      <c r="B77" s="2">
+        <v>2</v>
+      </c>
+      <c r="C77" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D77" s="27"/>
       <c r="E77" s="7"/>
       <c r="F77" s="2"/>
       <c r="G77" s="19"/>
       <c r="H77" s="2"/>
     </row>
     <row r="78" spans="1:8">
-      <c r="A78" s="42"/>
+      <c r="A78" s="98"/>
       <c r="B78" s="2"/>
-      <c r="C78" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="D78" s="28"/>
+      <c r="C78" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="D78" s="27"/>
       <c r="E78" s="7"/>
       <c r="F78" s="2"/>
       <c r="G78" s="19"/>
       <c r="H78" s="2"/>
     </row>
     <row r="79" spans="1:8">
-      <c r="A79" s="42"/>
+      <c r="A79" s="98"/>
       <c r="B79" s="2"/>
-      <c r="C79" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="D79" s="28"/>
+      <c r="C79" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="D79" s="27"/>
       <c r="E79" s="7"/>
       <c r="F79" s="2"/>
       <c r="G79" s="19"/>
       <c r="H79" s="2"/>
     </row>
     <row r="80" spans="1:8">
-      <c r="A80" s="42"/>
+      <c r="A80" s="98"/>
       <c r="B80" s="2"/>
-      <c r="C80" s="24"/>
-      <c r="D80" s="28"/>
+      <c r="C80" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="D80" s="27"/>
       <c r="E80" s="7"/>
       <c r="F80" s="2"/>
       <c r="G80" s="19"/>
       <c r="H80" s="2"/>
     </row>
     <row r="81" spans="1:8">
-      <c r="A81" s="42"/>
-      <c r="B81" s="2">
-        <v>3</v>
-      </c>
-      <c r="C81" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="D81" s="28"/>
+      <c r="A81" s="98"/>
+      <c r="B81" s="2"/>
+      <c r="C81" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="D81" s="27"/>
       <c r="E81" s="7"/>
       <c r="F81" s="2"/>
       <c r="G81" s="19"/>
       <c r="H81" s="2"/>
     </row>
     <row r="82" spans="1:8">
-      <c r="A82" s="42"/>
+      <c r="A82" s="98"/>
       <c r="B82" s="2"/>
-      <c r="C82" s="33" t="s">
-        <v>79</v>
-      </c>
-      <c r="D82" s="28"/>
+      <c r="C82" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="D82" s="27"/>
       <c r="E82" s="7"/>
       <c r="F82" s="2"/>
       <c r="G82" s="19"/>
       <c r="H82" s="2"/>
     </row>
     <row r="83" spans="1:8">
-      <c r="A83" s="42"/>
+      <c r="A83" s="98"/>
       <c r="B83" s="2"/>
-      <c r="C83" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="D83" s="28"/>
+      <c r="C83" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D83" s="27"/>
       <c r="E83" s="7"/>
       <c r="F83" s="2"/>
       <c r="G83" s="19"/>
       <c r="H83" s="2"/>
     </row>
     <row r="84" spans="1:8">
-      <c r="A84" s="42"/>
+      <c r="A84" s="98"/>
       <c r="B84" s="2"/>
-      <c r="C84" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="D84" s="28"/>
+      <c r="C84" s="24"/>
+      <c r="D84" s="27"/>
       <c r="E84" s="7"/>
       <c r="F84" s="2"/>
       <c r="G84" s="19"/>
       <c r="H84" s="2"/>
     </row>
     <row r="85" spans="1:8">
-      <c r="A85" s="42"/>
-      <c r="B85" s="2"/>
+      <c r="A85" s="98"/>
+      <c r="B85" s="2">
+        <v>3</v>
+      </c>
       <c r="C85" s="33" t="s">
-        <v>82</v>
-      </c>
-      <c r="D85" s="28"/>
+        <v>33</v>
+      </c>
+      <c r="D85" s="27"/>
       <c r="E85" s="7"/>
       <c r="F85" s="2"/>
       <c r="G85" s="19"/>
       <c r="H85" s="2"/>
     </row>
     <row r="86" spans="1:8">
-      <c r="A86" s="42"/>
+      <c r="A86" s="98"/>
       <c r="B86" s="2"/>
-      <c r="C86" s="33"/>
-      <c r="D86" s="28"/>
+      <c r="C86" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="D86" s="27"/>
       <c r="E86" s="7"/>
       <c r="F86" s="2"/>
       <c r="G86" s="19"/>
       <c r="H86" s="2"/>
     </row>
     <row r="87" spans="1:8">
-      <c r="A87" s="42"/>
-      <c r="B87" s="2">
-        <v>4</v>
-      </c>
-      <c r="C87" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D87" s="28"/>
+      <c r="A87" s="98"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="D87" s="27"/>
       <c r="E87" s="7"/>
       <c r="F87" s="2"/>
       <c r="G87" s="19"/>
       <c r="H87" s="2"/>
     </row>
     <row r="88" spans="1:8">
-      <c r="A88" s="42"/>
+      <c r="A88" s="98"/>
       <c r="B88" s="2"/>
-      <c r="C88" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="D88" s="28"/>
+      <c r="C88" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="D88" s="27"/>
       <c r="E88" s="7"/>
       <c r="F88" s="2"/>
       <c r="G88" s="19"/>
       <c r="H88" s="2"/>
     </row>
     <row r="89" spans="1:8">
-      <c r="A89" s="42"/>
+      <c r="A89" s="98"/>
       <c r="B89" s="2"/>
-      <c r="C89" s="33" t="s">
-        <v>83</v>
-      </c>
-      <c r="D89" s="28"/>
+      <c r="C89" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="D89" s="27"/>
       <c r="E89" s="7"/>
       <c r="F89" s="2"/>
       <c r="G89" s="19"/>
       <c r="H89" s="2"/>
     </row>
     <row r="90" spans="1:8">
-      <c r="A90" s="42"/>
+      <c r="A90" s="98"/>
       <c r="B90" s="2"/>
-      <c r="C90" s="33" t="s">
-        <v>84</v>
-      </c>
-      <c r="D90" s="28"/>
+      <c r="C90" s="28"/>
+      <c r="D90" s="27"/>
       <c r="E90" s="7"/>
       <c r="F90" s="2"/>
       <c r="G90" s="19"/>
       <c r="H90" s="2"/>
     </row>
     <row r="91" spans="1:8">
-      <c r="A91" s="42"/>
-      <c r="B91" s="2"/>
-      <c r="C91" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="D91" s="28"/>
+      <c r="A91" s="98"/>
+      <c r="B91" s="2">
+        <v>4</v>
+      </c>
+      <c r="C91" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D91" s="27"/>
       <c r="E91" s="7"/>
       <c r="F91" s="2"/>
       <c r="G91" s="19"/>
       <c r="H91" s="2"/>
     </row>
     <row r="92" spans="1:8">
-      <c r="A92" s="42"/>
+      <c r="A92" s="98"/>
       <c r="B92" s="2"/>
-      <c r="C92" s="33" t="s">
-        <v>82</v>
-      </c>
-      <c r="D92" s="28"/>
+      <c r="C92" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D92" s="27"/>
       <c r="E92" s="7"/>
       <c r="F92" s="2"/>
       <c r="G92" s="19"/>
       <c r="H92" s="2"/>
     </row>
     <row r="93" spans="1:8">
-      <c r="A93" s="42"/>
+      <c r="A93" s="98"/>
       <c r="B93" s="2"/>
-      <c r="C93" s="33"/>
-      <c r="D93" s="28"/>
+      <c r="C93" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D93" s="27"/>
       <c r="E93" s="7"/>
       <c r="F93" s="2"/>
       <c r="G93" s="19"/>
       <c r="H93" s="2"/>
     </row>
     <row r="94" spans="1:8">
-      <c r="A94" s="42"/>
+      <c r="A94" s="98"/>
       <c r="B94" s="2"/>
-      <c r="C94" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D94" s="28"/>
+      <c r="C94" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D94" s="27"/>
       <c r="E94" s="7"/>
       <c r="F94" s="2"/>
       <c r="G94" s="19"/>
       <c r="H94" s="2"/>
     </row>
     <row r="95" spans="1:8">
-      <c r="A95" s="42"/>
+      <c r="A95" s="98"/>
       <c r="B95" s="2"/>
-      <c r="C95" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="D95" s="28"/>
+      <c r="C95" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="D95" s="27"/>
       <c r="E95" s="7"/>
       <c r="F95" s="2"/>
       <c r="G95" s="19"/>
       <c r="H95" s="2"/>
     </row>
     <row r="96" spans="1:8">
-      <c r="A96" s="42"/>
+      <c r="A96" s="98"/>
       <c r="B96" s="2"/>
-      <c r="C96" s="33" t="s">
-        <v>87</v>
-      </c>
-      <c r="D96" s="28"/>
+      <c r="C96" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="D96" s="27"/>
       <c r="E96" s="7"/>
       <c r="F96" s="2"/>
       <c r="G96" s="19"/>
       <c r="H96" s="2"/>
     </row>
     <row r="97" spans="1:8">
-      <c r="A97" s="42"/>
+      <c r="A97" s="98"/>
       <c r="B97" s="2"/>
-      <c r="C97" s="33" t="s">
-        <v>88</v>
-      </c>
-      <c r="D97" s="28"/>
+      <c r="C97" s="28"/>
+      <c r="D97" s="27"/>
       <c r="E97" s="7"/>
       <c r="F97" s="2"/>
       <c r="G97" s="19"/>
       <c r="H97" s="2"/>
     </row>
     <row r="98" spans="1:8">
-      <c r="A98" s="42"/>
+      <c r="A98" s="98"/>
       <c r="B98" s="2"/>
-      <c r="C98" s="33" t="s">
-        <v>89</v>
-      </c>
-      <c r="D98" s="28"/>
+      <c r="C98" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="D98" s="27"/>
       <c r="E98" s="7"/>
       <c r="F98" s="2"/>
       <c r="G98" s="19"/>
       <c r="H98" s="2"/>
     </row>
     <row r="99" spans="1:8">
-      <c r="A99" s="42"/>
+      <c r="A99" s="98"/>
       <c r="B99" s="2"/>
-      <c r="C99" s="33" t="s">
-        <v>90</v>
-      </c>
-      <c r="D99" s="28"/>
+      <c r="C99" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="D99" s="27"/>
       <c r="E99" s="7"/>
       <c r="F99" s="2"/>
       <c r="G99" s="19"/>
       <c r="H99" s="2"/>
     </row>
     <row r="100" spans="1:8">
-      <c r="A100" s="42"/>
+      <c r="A100" s="98"/>
       <c r="B100" s="2"/>
-      <c r="C100" s="33"/>
-      <c r="D100" s="28"/>
+      <c r="C100" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="D100" s="27"/>
       <c r="E100" s="7"/>
       <c r="F100" s="2"/>
       <c r="G100" s="19"/>
       <c r="H100" s="2"/>
     </row>
     <row r="101" spans="1:8">
-      <c r="A101" s="42"/>
+      <c r="A101" s="98"/>
       <c r="B101" s="2"/>
-      <c r="C101" s="33"/>
-      <c r="D101" s="28"/>
+      <c r="C101" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="D101" s="27"/>
       <c r="E101" s="7"/>
       <c r="F101" s="2"/>
       <c r="G101" s="19"/>
       <c r="H101" s="2"/>
     </row>
     <row r="102" spans="1:8">
-      <c r="A102" s="42"/>
+      <c r="A102" s="98"/>
       <c r="B102" s="2"/>
-      <c r="C102" s="33"/>
-      <c r="D102" s="28"/>
+      <c r="C102" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="D102" s="27"/>
       <c r="E102" s="7"/>
       <c r="F102" s="2"/>
       <c r="G102" s="19"/>
       <c r="H102" s="2"/>
     </row>
     <row r="103" spans="1:8">
-      <c r="A103" s="42"/>
+      <c r="A103" s="98"/>
       <c r="B103" s="2"/>
-      <c r="C103" s="33"/>
-      <c r="D103" s="28"/>
+      <c r="C103" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D103" s="27"/>
       <c r="E103" s="7"/>
       <c r="F103" s="2"/>
       <c r="G103" s="19"/>
       <c r="H103" s="2"/>
     </row>
     <row r="104" spans="1:8">
-      <c r="A104" s="42"/>
+      <c r="A104" s="98"/>
       <c r="B104" s="2"/>
-      <c r="C104" s="33"/>
-      <c r="D104" s="28"/>
+      <c r="C104" s="28"/>
+      <c r="D104" s="27"/>
       <c r="E104" s="7"/>
       <c r="F104" s="2"/>
       <c r="G104" s="19"/>
       <c r="H104" s="2"/>
     </row>
     <row r="105" spans="1:8">
-      <c r="A105" s="42"/>
+      <c r="A105" s="98"/>
       <c r="B105" s="2"/>
-      <c r="C105" s="24"/>
-      <c r="D105" s="13"/>
+      <c r="C105" s="28"/>
+      <c r="D105" s="27"/>
       <c r="E105" s="7"/>
       <c r="F105" s="2"/>
       <c r="G105" s="19"/>
       <c r="H105" s="2"/>
     </row>
     <row r="106" spans="1:8">
-      <c r="A106" s="42"/>
+      <c r="A106" s="98"/>
       <c r="B106" s="2"/>
-      <c r="C106" s="24"/>
-      <c r="D106" s="13"/>
+      <c r="C106" s="28"/>
+      <c r="D106" s="27"/>
       <c r="E106" s="7"/>
       <c r="F106" s="2"/>
       <c r="G106" s="19"/>
       <c r="H106" s="2"/>
     </row>
     <row r="107" spans="1:8">
-      <c r="A107" s="42"/>
+      <c r="A107" s="98"/>
       <c r="B107" s="2"/>
-      <c r="C107" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D107" s="13"/>
+      <c r="C107" s="28"/>
+      <c r="D107" s="27"/>
       <c r="E107" s="7"/>
       <c r="F107" s="2"/>
       <c r="G107" s="19"/>
       <c r="H107" s="2"/>
     </row>
     <row r="108" spans="1:8">
-      <c r="A108" s="42"/>
+      <c r="A108" s="98"/>
       <c r="B108" s="2"/>
-      <c r="C108" s="37"/>
-      <c r="D108" s="13"/>
+      <c r="C108" s="28"/>
+      <c r="D108" s="27"/>
       <c r="E108" s="7"/>
       <c r="F108" s="2"/>
       <c r="G108" s="19"/>
       <c r="H108" s="2"/>
     </row>
     <row r="109" spans="1:8">
-      <c r="A109" s="42"/>
+      <c r="A109" s="98"/>
       <c r="B109" s="2"/>
-      <c r="C109" s="38" t="s">
-        <v>34</v>
-      </c>
-      <c r="D109" s="25" t="s">
-        <v>11</v>
-      </c>
+      <c r="C109" s="24"/>
+      <c r="D109" s="13"/>
       <c r="E109" s="7"/>
       <c r="F109" s="2"/>
       <c r="G109" s="19"/>
       <c r="H109" s="2"/>
     </row>
     <row r="110" spans="1:8">
-      <c r="A110" s="42"/>
+      <c r="A110" s="98"/>
       <c r="B110" s="2"/>
-      <c r="C110" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="D110" s="25"/>
+      <c r="C110" s="24"/>
+      <c r="D110" s="13"/>
       <c r="E110" s="7"/>
       <c r="F110" s="2"/>
       <c r="G110" s="19"/>
       <c r="H110" s="2"/>
     </row>
     <row r="111" spans="1:8">
-      <c r="A111" s="42"/>
+      <c r="A111" s="98"/>
       <c r="B111" s="2"/>
-      <c r="C111" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="D111" s="25"/>
+      <c r="C111" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="D111" s="13"/>
       <c r="E111" s="7"/>
       <c r="F111" s="2"/>
       <c r="G111" s="19"/>
       <c r="H111" s="2"/>
     </row>
     <row r="112" spans="1:8">
-      <c r="A112" s="42"/>
+      <c r="A112" s="98"/>
       <c r="B112" s="2"/>
-      <c r="C112" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="D112" s="25"/>
+      <c r="C112" s="31"/>
+      <c r="D112" s="13"/>
       <c r="E112" s="7"/>
       <c r="F112" s="2"/>
       <c r="G112" s="19"/>
       <c r="H112" s="2"/>
     </row>
     <row r="113" spans="1:8">
-      <c r="A113" s="42"/>
+      <c r="A113" s="98"/>
       <c r="B113" s="2"/>
-      <c r="C113" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="D113" s="25"/>
+      <c r="C113" s="74" t="s">
+        <v>30</v>
+      </c>
+      <c r="D113" s="25" t="s">
+        <v>10</v>
+      </c>
       <c r="E113" s="7"/>
-      <c r="F113" s="2"/>
+      <c r="F113" s="84" t="s">
+        <v>113</v>
+      </c>
       <c r="G113" s="19"/>
       <c r="H113" s="2"/>
     </row>
     <row r="114" spans="1:8">
-      <c r="A114" s="42"/>
+      <c r="A114" s="98"/>
       <c r="B114" s="2"/>
-      <c r="C114" s="29"/>
+      <c r="C114" s="71" t="s">
+        <v>56</v>
+      </c>
       <c r="D114" s="25"/>
       <c r="E114" s="7"/>
       <c r="F114" s="2"/>
@@ -2452,10 +2717,10 @@
       <c r="H114" s="2"/>
     </row>
     <row r="115" spans="1:8">
-      <c r="A115" s="42"/>
+      <c r="A115" s="98"/>
       <c r="B115" s="2"/>
-      <c r="C115" s="38" t="s">
-        <v>67</v>
+      <c r="C115" s="72" t="s">
+        <v>57</v>
       </c>
       <c r="D115" s="25"/>
       <c r="E115" s="7"/>
@@ -2464,10 +2729,10 @@
       <c r="H115" s="2"/>
     </row>
     <row r="116" spans="1:8">
-      <c r="A116" s="42"/>
+      <c r="A116" s="98"/>
       <c r="B116" s="2"/>
-      <c r="C116" s="29" t="s">
-        <v>68</v>
+      <c r="C116" s="72" t="s">
+        <v>58</v>
       </c>
       <c r="D116" s="25"/>
       <c r="E116" s="7"/>
@@ -2476,10 +2741,10 @@
       <c r="H116" s="2"/>
     </row>
     <row r="117" spans="1:8">
-      <c r="A117" s="42"/>
+      <c r="A117" s="98"/>
       <c r="B117" s="2"/>
-      <c r="C117" s="29" t="s">
-        <v>69</v>
+      <c r="C117" s="72" t="s">
+        <v>59</v>
       </c>
       <c r="D117" s="25"/>
       <c r="E117" s="7"/>
@@ -2488,53 +2753,57 @@
       <c r="H117" s="2"/>
     </row>
     <row r="118" spans="1:8">
-      <c r="A118" s="42"/>
+      <c r="A118" s="98"/>
       <c r="B118" s="2"/>
-      <c r="C118" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="D118" s="13"/>
+      <c r="C118" s="72"/>
+      <c r="D118" s="25"/>
       <c r="E118" s="7"/>
       <c r="F118" s="2"/>
       <c r="G118" s="19"/>
       <c r="H118" s="2"/>
     </row>
     <row r="119" spans="1:8">
-      <c r="A119" s="42"/>
+      <c r="A119" s="98"/>
       <c r="B119" s="2"/>
-      <c r="C119" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="D119" s="13"/>
+      <c r="C119" s="71" t="s">
+        <v>60</v>
+      </c>
+      <c r="D119" s="25"/>
       <c r="E119" s="7"/>
       <c r="F119" s="2"/>
       <c r="G119" s="19"/>
       <c r="H119" s="2"/>
     </row>
     <row r="120" spans="1:8">
-      <c r="A120" s="42"/>
+      <c r="A120" s="98"/>
       <c r="B120" s="2"/>
-      <c r="C120" s="24"/>
-      <c r="D120" s="13"/>
+      <c r="C120" s="72" t="s">
+        <v>61</v>
+      </c>
+      <c r="D120" s="25"/>
       <c r="E120" s="7"/>
       <c r="F120" s="2"/>
       <c r="G120" s="19"/>
       <c r="H120" s="2"/>
     </row>
     <row r="121" spans="1:8">
-      <c r="A121" s="42"/>
+      <c r="A121" s="98"/>
       <c r="B121" s="2"/>
-      <c r="C121" s="24"/>
-      <c r="D121" s="13"/>
+      <c r="C121" s="72" t="s">
+        <v>62</v>
+      </c>
+      <c r="D121" s="25"/>
       <c r="E121" s="7"/>
       <c r="F121" s="2"/>
       <c r="G121" s="19"/>
       <c r="H121" s="2"/>
     </row>
     <row r="122" spans="1:8">
-      <c r="A122" s="42"/>
+      <c r="A122" s="98"/>
       <c r="B122" s="2"/>
-      <c r="C122" s="24"/>
+      <c r="C122" s="70" t="s">
+        <v>63</v>
+      </c>
       <c r="D122" s="13"/>
       <c r="E122" s="7"/>
       <c r="F122" s="2"/>
@@ -2542,9 +2811,11 @@
       <c r="H122" s="2"/>
     </row>
     <row r="123" spans="1:8">
-      <c r="A123" s="42"/>
+      <c r="A123" s="98"/>
       <c r="B123" s="2"/>
-      <c r="C123" s="24"/>
+      <c r="C123" s="24" t="s">
+        <v>64</v>
+      </c>
       <c r="D123" s="13"/>
       <c r="E123" s="7"/>
       <c r="F123" s="2"/>
@@ -2552,11 +2823,9 @@
       <c r="H123" s="2"/>
     </row>
     <row r="124" spans="1:8">
-      <c r="A124" s="42"/>
+      <c r="A124" s="98"/>
       <c r="B124" s="2"/>
-      <c r="C124" s="14" t="s">
-        <v>39</v>
-      </c>
+      <c r="C124" s="24"/>
       <c r="D124" s="13"/>
       <c r="E124" s="7"/>
       <c r="F124" s="2"/>
@@ -2564,9 +2833,9 @@
       <c r="H124" s="2"/>
     </row>
     <row r="125" spans="1:8">
-      <c r="A125" s="42"/>
+      <c r="A125" s="98"/>
       <c r="B125" s="2"/>
-      <c r="C125" s="37"/>
+      <c r="C125" s="24"/>
       <c r="D125" s="13"/>
       <c r="E125" s="7"/>
       <c r="F125" s="2"/>
@@ -2574,25 +2843,19 @@
       <c r="H125" s="2"/>
     </row>
     <row r="126" spans="1:8">
-      <c r="A126" s="42"/>
+      <c r="A126" s="98"/>
       <c r="B126" s="2"/>
-      <c r="C126" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="D126" s="34" t="s">
-        <v>11</v>
-      </c>
+      <c r="C126" s="24"/>
+      <c r="D126" s="13"/>
       <c r="E126" s="7"/>
       <c r="F126" s="2"/>
       <c r="G126" s="19"/>
       <c r="H126" s="2"/>
     </row>
     <row r="127" spans="1:8">
-      <c r="A127" s="42"/>
+      <c r="A127" s="98"/>
       <c r="B127" s="2"/>
-      <c r="C127" s="33" t="s">
-        <v>58</v>
-      </c>
+      <c r="C127" s="24"/>
       <c r="D127" s="13"/>
       <c r="E127" s="7"/>
       <c r="F127" s="2"/>
@@ -2600,10 +2863,10 @@
       <c r="H127" s="2"/>
     </row>
     <row r="128" spans="1:8">
-      <c r="A128" s="42"/>
+      <c r="A128" s="98"/>
       <c r="B128" s="2"/>
-      <c r="C128" s="33" t="s">
-        <v>57</v>
+      <c r="C128" s="14" t="s">
+        <v>125</v>
       </c>
       <c r="D128" s="13"/>
       <c r="E128" s="7"/>
@@ -2612,9 +2875,9 @@
       <c r="H128" s="2"/>
     </row>
     <row r="129" spans="1:8">
-      <c r="A129" s="42"/>
+      <c r="A129" s="98"/>
       <c r="B129" s="2"/>
-      <c r="C129" s="24"/>
+      <c r="C129" s="31"/>
       <c r="D129" s="13"/>
       <c r="E129" s="7"/>
       <c r="F129" s="2"/>
@@ -2622,34 +2885,38 @@
       <c r="H129" s="2"/>
     </row>
     <row r="130" spans="1:8">
-      <c r="A130" s="42"/>
+      <c r="A130" s="98"/>
       <c r="B130" s="2"/>
-      <c r="C130" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="D130" s="13"/>
+      <c r="C130" s="75" t="s">
+        <v>45</v>
+      </c>
+      <c r="D130" s="29" t="s">
+        <v>10</v>
+      </c>
       <c r="E130" s="7"/>
-      <c r="F130" s="2"/>
+      <c r="F130" s="62" t="s">
+        <v>114</v>
+      </c>
       <c r="G130" s="19"/>
       <c r="H130" s="2"/>
     </row>
     <row r="131" spans="1:8">
-      <c r="A131" s="42"/>
+      <c r="A131" s="98"/>
       <c r="B131" s="2"/>
-      <c r="C131" s="33" t="s">
-        <v>60</v>
+      <c r="C131" s="28" t="s">
+        <v>51</v>
       </c>
       <c r="D131" s="13"/>
       <c r="E131" s="7"/>
-      <c r="F131" s="2"/>
+      <c r="F131" s="34"/>
       <c r="G131" s="19"/>
       <c r="H131" s="2"/>
     </row>
     <row r="132" spans="1:8">
-      <c r="A132" s="42"/>
+      <c r="A132" s="98"/>
       <c r="B132" s="2"/>
-      <c r="C132" s="33" t="s">
-        <v>61</v>
+      <c r="C132" s="28" t="s">
+        <v>50</v>
       </c>
       <c r="D132" s="13"/>
       <c r="E132" s="7"/>
@@ -2658,11 +2925,9 @@
       <c r="H132" s="2"/>
     </row>
     <row r="133" spans="1:8">
-      <c r="A133" s="42"/>
+      <c r="A133" s="98"/>
       <c r="B133" s="2"/>
-      <c r="C133" s="33" t="s">
-        <v>62</v>
-      </c>
+      <c r="C133" s="24"/>
       <c r="D133" s="13"/>
       <c r="E133" s="7"/>
       <c r="F133" s="2"/>
@@ -2670,9 +2935,11 @@
       <c r="H133" s="2"/>
     </row>
     <row r="134" spans="1:8">
-      <c r="A134" s="42"/>
+      <c r="A134" s="98"/>
       <c r="B134" s="2"/>
-      <c r="C134" s="24"/>
+      <c r="C134" s="30" t="s">
+        <v>52</v>
+      </c>
       <c r="D134" s="13"/>
       <c r="E134" s="7"/>
       <c r="F134" s="2"/>
@@ -2680,9 +2947,11 @@
       <c r="H134" s="2"/>
     </row>
     <row r="135" spans="1:8">
-      <c r="A135" s="43"/>
+      <c r="A135" s="98"/>
       <c r="B135" s="2"/>
-      <c r="C135" s="16"/>
+      <c r="C135" s="28" t="s">
+        <v>53</v>
+      </c>
       <c r="D135" s="13"/>
       <c r="E135" s="7"/>
       <c r="F135" s="2"/>
@@ -2690,33 +2959,33 @@
       <c r="H135" s="2"/>
     </row>
     <row r="136" spans="1:8">
-      <c r="A136" s="3"/>
-      <c r="B136" s="5"/>
-      <c r="C136" s="9"/>
-      <c r="D136" s="5"/>
-      <c r="E136" s="9"/>
-      <c r="F136" s="5"/>
-      <c r="G136" s="21"/>
-      <c r="H136" s="5"/>
+      <c r="A136" s="98"/>
+      <c r="B136" s="2"/>
+      <c r="C136" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D136" s="13"/>
+      <c r="E136" s="7"/>
+      <c r="F136" s="2"/>
+      <c r="G136" s="19"/>
+      <c r="H136" s="2"/>
     </row>
     <row r="137" spans="1:8">
-      <c r="A137" s="41" t="s">
-        <v>9</v>
-      </c>
+      <c r="A137" s="98"/>
       <c r="B137" s="2"/>
-      <c r="C137" s="16"/>
+      <c r="C137" s="28" t="s">
+        <v>55</v>
+      </c>
       <c r="D137" s="13"/>
       <c r="E137" s="7"/>
-      <c r="F137" s="17"/>
+      <c r="F137" s="2"/>
       <c r="G137" s="19"/>
       <c r="H137" s="2"/>
     </row>
     <row r="138" spans="1:8">
-      <c r="A138" s="42"/>
+      <c r="A138" s="98"/>
       <c r="B138" s="2"/>
-      <c r="C138" s="14" t="s">
-        <v>22</v>
-      </c>
+      <c r="C138" s="24"/>
       <c r="D138" s="13"/>
       <c r="E138" s="7"/>
       <c r="F138" s="2"/>
@@ -2724,42 +2993,42 @@
       <c r="H138" s="2"/>
     </row>
     <row r="139" spans="1:8">
-      <c r="A139" s="42"/>
+      <c r="A139" s="99"/>
       <c r="B139" s="2"/>
-      <c r="C139" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="D139" s="23"/>
+      <c r="C139" s="16"/>
+      <c r="D139" s="13"/>
       <c r="E139" s="7"/>
       <c r="F139" s="2"/>
       <c r="G139" s="19"/>
       <c r="H139" s="2"/>
     </row>
     <row r="140" spans="1:8">
-      <c r="A140" s="42"/>
-      <c r="B140" s="2"/>
-      <c r="C140" s="16"/>
-      <c r="D140" s="23"/>
-      <c r="E140" s="7"/>
-      <c r="F140" s="2"/>
-      <c r="G140" s="19"/>
-      <c r="H140" s="2"/>
+      <c r="A140" s="3"/>
+      <c r="B140" s="5"/>
+      <c r="C140" s="9"/>
+      <c r="D140" s="5"/>
+      <c r="E140" s="9"/>
+      <c r="F140" s="5"/>
+      <c r="G140" s="21"/>
+      <c r="H140" s="5"/>
     </row>
     <row r="141" spans="1:8">
-      <c r="A141" s="42"/>
+      <c r="A141" s="97" t="s">
+        <v>101</v>
+      </c>
       <c r="B141" s="2"/>
       <c r="C141" s="16"/>
       <c r="D141" s="13"/>
       <c r="E141" s="7"/>
-      <c r="F141" s="2"/>
+      <c r="F141" s="17"/>
       <c r="G141" s="19"/>
       <c r="H141" s="2"/>
     </row>
     <row r="142" spans="1:8">
-      <c r="A142" s="42"/>
+      <c r="A142" s="98"/>
       <c r="B142" s="2"/>
       <c r="C142" s="14" t="s">
-        <v>38</v>
+        <v>124</v>
       </c>
       <c r="D142" s="13"/>
       <c r="E142" s="7"/>
@@ -2768,185 +3037,211 @@
       <c r="H142" s="2"/>
     </row>
     <row r="143" spans="1:8">
-      <c r="A143" s="42"/>
+      <c r="A143" s="98"/>
       <c r="B143" s="2"/>
       <c r="C143" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="D143" s="17"/>
+        <v>28</v>
+      </c>
+      <c r="D143" s="23"/>
       <c r="E143" s="7"/>
-      <c r="F143" s="17"/>
+      <c r="F143" s="2"/>
       <c r="G143" s="19"/>
       <c r="H143" s="2"/>
     </row>
     <row r="144" spans="1:8">
-      <c r="A144" s="42"/>
+      <c r="A144" s="98"/>
       <c r="B144" s="2"/>
       <c r="C144" s="16"/>
-      <c r="D144" s="17"/>
+      <c r="D144" s="23"/>
       <c r="E144" s="7"/>
-      <c r="F144" s="17"/>
+      <c r="F144" s="2"/>
       <c r="G144" s="19"/>
       <c r="H144" s="2"/>
     </row>
     <row r="145" spans="1:8">
-      <c r="A145" s="42"/>
+      <c r="A145" s="98"/>
       <c r="B145" s="2"/>
-      <c r="C145" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="D145" s="17"/>
+      <c r="C145" s="16"/>
+      <c r="D145" s="13"/>
       <c r="E145" s="7"/>
-      <c r="F145" s="17"/>
+      <c r="F145" s="2"/>
       <c r="G145" s="19"/>
       <c r="H145" s="2"/>
     </row>
     <row r="146" spans="1:8">
-      <c r="A146" s="42"/>
+      <c r="A146" s="98"/>
       <c r="B146" s="2"/>
-      <c r="C146" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="D146" s="17"/>
+      <c r="C146" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="D146" s="13"/>
       <c r="E146" s="7"/>
-      <c r="F146" s="17"/>
+      <c r="F146" s="2"/>
       <c r="G146" s="19"/>
       <c r="H146" s="2"/>
     </row>
     <row r="147" spans="1:8">
-      <c r="A147" s="42"/>
+      <c r="A147" s="98"/>
       <c r="B147" s="2"/>
-      <c r="C147" s="16"/>
-      <c r="D147" s="2"/>
+      <c r="C147" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="D147" s="17"/>
       <c r="E147" s="7"/>
-      <c r="F147" s="2"/>
+      <c r="F147" s="17"/>
       <c r="G147" s="19"/>
       <c r="H147" s="2"/>
     </row>
     <row r="148" spans="1:8">
-      <c r="A148" s="43"/>
+      <c r="A148" s="98"/>
       <c r="B148" s="2"/>
-      <c r="C148" s="7"/>
-      <c r="D148" s="2"/>
+      <c r="C148" s="16"/>
+      <c r="D148" s="17"/>
       <c r="E148" s="7"/>
-      <c r="F148" s="2"/>
+      <c r="F148" s="17"/>
       <c r="G148" s="19"/>
       <c r="H148" s="2"/>
     </row>
     <row r="149" spans="1:8">
-      <c r="A149" s="3"/>
-      <c r="B149" s="5"/>
-      <c r="C149" s="9"/>
-      <c r="D149" s="5"/>
-      <c r="E149" s="9"/>
-      <c r="F149" s="5"/>
-      <c r="G149" s="21"/>
-      <c r="H149" s="5"/>
+      <c r="A149" s="98"/>
+      <c r="B149" s="2"/>
+      <c r="C149" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="D149" s="17"/>
+      <c r="E149" s="7"/>
+      <c r="F149" s="17"/>
+      <c r="G149" s="19"/>
+      <c r="H149" s="2"/>
     </row>
     <row r="150" spans="1:8">
-      <c r="A150" s="41" t="s">
-        <v>10</v>
-      </c>
+      <c r="A150" s="98"/>
       <c r="B150" s="2"/>
-      <c r="C150" s="7"/>
-      <c r="D150" s="2"/>
+      <c r="C150" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="D150" s="17"/>
       <c r="E150" s="7"/>
-      <c r="F150" s="2"/>
+      <c r="F150" s="17"/>
       <c r="G150" s="19"/>
       <c r="H150" s="2"/>
     </row>
     <row r="151" spans="1:8">
-      <c r="A151" s="42"/>
-      <c r="B151" s="2"/>
-      <c r="C151" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D151" s="2"/>
-      <c r="E151" s="7"/>
-      <c r="F151" s="2"/>
-      <c r="G151" s="19"/>
-      <c r="H151" s="2"/>
-    </row>
-    <row r="152" spans="1:8">
-      <c r="A152" s="42"/>
-      <c r="B152" s="2"/>
-      <c r="C152" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D152" s="2"/>
-      <c r="E152" s="7"/>
-      <c r="F152" s="2"/>
-      <c r="G152" s="19"/>
-      <c r="H152" s="2"/>
+      <c r="A151" s="98"/>
+      <c r="B151" s="44"/>
+      <c r="C151" s="45"/>
+      <c r="D151" s="46"/>
+      <c r="E151" s="47"/>
+      <c r="F151" s="46"/>
+      <c r="G151" s="48"/>
+      <c r="H151" s="44"/>
+    </row>
+    <row r="152" spans="1:8" s="57" customFormat="1">
+      <c r="A152" s="98"/>
+      <c r="C152" s="58"/>
+      <c r="D152" s="59"/>
+      <c r="E152" s="60"/>
+      <c r="F152" s="59"/>
+      <c r="G152" s="61"/>
     </row>
     <row r="153" spans="1:8">
-      <c r="A153" s="42"/>
-      <c r="B153" s="2"/>
-      <c r="C153" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D153" s="2"/>
-      <c r="E153" s="7"/>
-      <c r="F153" s="2"/>
-      <c r="G153" s="19"/>
-      <c r="H153" s="2"/>
-    </row>
-    <row r="154" spans="1:8">
-      <c r="A154" s="42"/>
+      <c r="A153" s="98"/>
+      <c r="B153" s="49"/>
+      <c r="C153" s="50"/>
+      <c r="D153" s="51"/>
+      <c r="E153" s="52"/>
+      <c r="F153" s="51"/>
+      <c r="G153" s="53"/>
+      <c r="H153" s="85"/>
+    </row>
+    <row r="154" spans="1:8" ht="43.5">
+      <c r="A154" s="98"/>
       <c r="B154" s="2"/>
-      <c r="C154" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D154" s="2"/>
+      <c r="C154" s="62" t="s">
+        <v>92</v>
+      </c>
+      <c r="D154" s="54" t="s">
+        <v>93</v>
+      </c>
       <c r="E154" s="7"/>
-      <c r="F154" s="2"/>
-      <c r="G154" s="19"/>
-      <c r="H154" s="2"/>
-    </row>
-    <row r="155" spans="1:8">
-      <c r="A155" s="42"/>
+      <c r="F154" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="G154" s="55" t="s">
+        <v>100</v>
+      </c>
+      <c r="H154" s="86" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" ht="43.5">
+      <c r="A155" s="98"/>
       <c r="B155" s="2"/>
-      <c r="C155" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D155" s="2"/>
+      <c r="C155" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="D155" s="67" t="s">
+        <v>111</v>
+      </c>
       <c r="E155" s="7"/>
-      <c r="F155" s="2"/>
-      <c r="G155" s="19"/>
-      <c r="H155" s="2"/>
-    </row>
-    <row r="156" spans="1:8">
-      <c r="A156" s="42"/>
+      <c r="F155" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="G155" s="55" t="s">
+        <v>97</v>
+      </c>
+      <c r="H155" s="86" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" ht="43.5">
+      <c r="A156" s="98"/>
       <c r="B156" s="2"/>
-      <c r="C156" s="7"/>
-      <c r="D156" s="2"/>
+      <c r="C156" s="62" t="s">
+        <v>98</v>
+      </c>
+      <c r="D156" s="54" t="s">
+        <v>95</v>
+      </c>
       <c r="E156" s="7"/>
-      <c r="F156" s="2"/>
-      <c r="G156" s="19"/>
-      <c r="H156" s="2"/>
+      <c r="F156" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="G156" s="55" t="s">
+        <v>100</v>
+      </c>
+      <c r="H156" s="86" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="157" spans="1:8">
-      <c r="A157" s="42"/>
+      <c r="A157" s="98"/>
       <c r="B157" s="2"/>
-      <c r="C157" s="7"/>
-      <c r="D157" s="2"/>
+      <c r="C157" s="34"/>
+      <c r="D157" s="17"/>
       <c r="E157" s="7"/>
-      <c r="F157" s="2"/>
+      <c r="F157" s="17"/>
       <c r="G157" s="19"/>
-      <c r="H157" s="2"/>
+      <c r="H157" s="49"/>
     </row>
     <row r="158" spans="1:8">
-      <c r="A158" s="42"/>
+      <c r="A158" s="98"/>
       <c r="B158" s="2"/>
-      <c r="C158" s="7"/>
-      <c r="D158" s="2"/>
+      <c r="C158" s="100" t="s">
+        <v>122</v>
+      </c>
+      <c r="D158" s="63" t="s">
+        <v>32</v>
+      </c>
       <c r="E158" s="7"/>
-      <c r="F158" s="2"/>
+      <c r="F158" s="63" t="s">
+        <v>110</v>
+      </c>
       <c r="G158" s="19"/>
       <c r="H158" s="2"/>
     </row>
     <row r="159" spans="1:8">
-      <c r="A159" s="42"/>
+      <c r="A159" s="99"/>
       <c r="B159" s="2"/>
       <c r="C159" s="7"/>
       <c r="D159" s="2"/>
@@ -2956,17 +3251,19 @@
       <c r="H159" s="2"/>
     </row>
     <row r="160" spans="1:8">
-      <c r="A160" s="42"/>
-      <c r="B160" s="2"/>
-      <c r="C160" s="7"/>
-      <c r="D160" s="2"/>
-      <c r="E160" s="7"/>
-      <c r="F160" s="2"/>
-      <c r="G160" s="19"/>
-      <c r="H160" s="2"/>
+      <c r="A160" s="3"/>
+      <c r="B160" s="5"/>
+      <c r="C160" s="9"/>
+      <c r="D160" s="5"/>
+      <c r="E160" s="9"/>
+      <c r="F160" s="5"/>
+      <c r="G160" s="21"/>
+      <c r="H160" s="5"/>
     </row>
     <row r="161" spans="1:8">
-      <c r="A161" s="42"/>
+      <c r="A161" s="97" t="s">
+        <v>9</v>
+      </c>
       <c r="B161" s="2"/>
       <c r="C161" s="7"/>
       <c r="D161" s="2"/>
@@ -2976,9 +3273,11 @@
       <c r="H161" s="2"/>
     </row>
     <row r="162" spans="1:8">
-      <c r="A162" s="42"/>
+      <c r="A162" s="98"/>
       <c r="B162" s="2"/>
-      <c r="C162" s="7"/>
+      <c r="C162" s="7" t="s">
+        <v>11</v>
+      </c>
       <c r="D162" s="2"/>
       <c r="E162" s="7"/>
       <c r="F162" s="2"/>
@@ -2986,9 +3285,11 @@
       <c r="H162" s="2"/>
     </row>
     <row r="163" spans="1:8">
-      <c r="A163" s="42"/>
+      <c r="A163" s="98"/>
       <c r="B163" s="2"/>
-      <c r="C163" s="7"/>
+      <c r="C163" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="D163" s="2"/>
       <c r="E163" s="7"/>
       <c r="F163" s="2"/>
@@ -2996,9 +3297,11 @@
       <c r="H163" s="2"/>
     </row>
     <row r="164" spans="1:8">
-      <c r="A164" s="42"/>
+      <c r="A164" s="98"/>
       <c r="B164" s="2"/>
-      <c r="C164" s="7"/>
+      <c r="C164" s="7" t="s">
+        <v>13</v>
+      </c>
       <c r="D164" s="2"/>
       <c r="E164" s="7"/>
       <c r="F164" s="2"/>
@@ -3006,9 +3309,11 @@
       <c r="H164" s="2"/>
     </row>
     <row r="165" spans="1:8">
-      <c r="A165" s="42"/>
+      <c r="A165" s="98"/>
       <c r="B165" s="2"/>
-      <c r="C165" s="7"/>
+      <c r="C165" s="7" t="s">
+        <v>14</v>
+      </c>
       <c r="D165" s="2"/>
       <c r="E165" s="7"/>
       <c r="F165" s="2"/>
@@ -3016,9 +3321,11 @@
       <c r="H165" s="2"/>
     </row>
     <row r="166" spans="1:8">
-      <c r="A166" s="42"/>
+      <c r="A166" s="98"/>
       <c r="B166" s="2"/>
-      <c r="C166" s="7"/>
+      <c r="C166" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="D166" s="2"/>
       <c r="E166" s="7"/>
       <c r="F166" s="2"/>
@@ -3026,9 +3333,11 @@
       <c r="H166" s="2"/>
     </row>
     <row r="167" spans="1:8">
-      <c r="A167" s="42"/>
+      <c r="A167" s="98"/>
       <c r="B167" s="2"/>
-      <c r="C167" s="7"/>
+      <c r="C167" s="67" t="s">
+        <v>104</v>
+      </c>
       <c r="D167" s="2"/>
       <c r="E167" s="7"/>
       <c r="F167" s="2"/>
@@ -3036,36 +3345,147 @@
       <c r="H167" s="2"/>
     </row>
     <row r="168" spans="1:8">
-      <c r="A168" s="3"/>
-      <c r="B168" s="4"/>
-      <c r="C168" s="8"/>
-      <c r="D168" s="4"/>
-      <c r="E168" s="8"/>
-      <c r="F168" s="4"/>
-      <c r="G168" s="20"/>
-      <c r="H168" s="4"/>
+      <c r="A168" s="98"/>
+      <c r="B168" s="2"/>
+      <c r="C168" s="7"/>
+      <c r="D168" s="2"/>
+      <c r="E168" s="7"/>
+      <c r="F168" s="2"/>
+      <c r="G168" s="19"/>
+      <c r="H168" s="2"/>
+    </row>
+    <row r="169" spans="1:8">
+      <c r="A169" s="98"/>
+      <c r="B169" s="2"/>
+      <c r="C169" s="7"/>
+      <c r="D169" s="2"/>
+      <c r="E169" s="7"/>
+      <c r="F169" s="2"/>
+      <c r="G169" s="19"/>
+      <c r="H169" s="2"/>
+    </row>
+    <row r="170" spans="1:8">
+      <c r="A170" s="98"/>
+      <c r="B170" s="2"/>
+      <c r="C170" s="7"/>
+      <c r="D170" s="2"/>
+      <c r="E170" s="7"/>
+      <c r="F170" s="2"/>
+      <c r="G170" s="19"/>
+      <c r="H170" s="2"/>
+    </row>
+    <row r="171" spans="1:8">
+      <c r="A171" s="98"/>
+      <c r="B171" s="2"/>
+      <c r="C171" s="7"/>
+      <c r="D171" s="2"/>
+      <c r="E171" s="7"/>
+      <c r="F171" s="2"/>
+      <c r="G171" s="19"/>
+      <c r="H171" s="2"/>
+    </row>
+    <row r="172" spans="1:8">
+      <c r="A172" s="98"/>
+      <c r="B172" s="2"/>
+      <c r="C172" s="7"/>
+      <c r="D172" s="2"/>
+      <c r="E172" s="7"/>
+      <c r="F172" s="2"/>
+      <c r="G172" s="19"/>
+      <c r="H172" s="2"/>
+    </row>
+    <row r="173" spans="1:8">
+      <c r="A173" s="98"/>
+      <c r="B173" s="2"/>
+      <c r="C173" s="7"/>
+      <c r="D173" s="2"/>
+      <c r="E173" s="7"/>
+      <c r="F173" s="2"/>
+      <c r="G173" s="19"/>
+      <c r="H173" s="2"/>
+    </row>
+    <row r="174" spans="1:8">
+      <c r="A174" s="98"/>
+      <c r="B174" s="2"/>
+      <c r="C174" s="7"/>
+      <c r="D174" s="2"/>
+      <c r="E174" s="7"/>
+      <c r="F174" s="2"/>
+      <c r="G174" s="19"/>
+      <c r="H174" s="2"/>
+    </row>
+    <row r="175" spans="1:8">
+      <c r="A175" s="98"/>
+      <c r="B175" s="2"/>
+      <c r="C175" s="7"/>
+      <c r="D175" s="2"/>
+      <c r="E175" s="7"/>
+      <c r="F175" s="2"/>
+      <c r="G175" s="19"/>
+      <c r="H175" s="2"/>
+    </row>
+    <row r="176" spans="1:8">
+      <c r="A176" s="98"/>
+      <c r="B176" s="2"/>
+      <c r="C176" s="7"/>
+      <c r="D176" s="2"/>
+      <c r="E176" s="7"/>
+      <c r="F176" s="2"/>
+      <c r="G176" s="19"/>
+      <c r="H176" s="2"/>
+    </row>
+    <row r="177" spans="1:8">
+      <c r="A177" s="98"/>
+      <c r="B177" s="2"/>
+      <c r="C177" s="7"/>
+      <c r="D177" s="2"/>
+      <c r="E177" s="7"/>
+      <c r="F177" s="2"/>
+      <c r="G177" s="19"/>
+      <c r="H177" s="2"/>
+    </row>
+    <row r="178" spans="1:8">
+      <c r="A178" s="98"/>
+      <c r="B178" s="2"/>
+      <c r="C178" s="7"/>
+      <c r="D178" s="2"/>
+      <c r="E178" s="7"/>
+      <c r="F178" s="2"/>
+      <c r="G178" s="19"/>
+      <c r="H178" s="2"/>
+    </row>
+    <row r="179" spans="1:8">
+      <c r="A179" s="3"/>
+      <c r="B179" s="4"/>
+      <c r="C179" s="8"/>
+      <c r="D179" s="4"/>
+      <c r="E179" s="8"/>
+      <c r="F179" s="4"/>
+      <c r="G179" s="20"/>
+      <c r="H179" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A150:A167"/>
-    <mergeCell ref="A2:A16"/>
-    <mergeCell ref="A18:A58"/>
-    <mergeCell ref="A60:A135"/>
-    <mergeCell ref="A137:A148"/>
+    <mergeCell ref="A161:A178"/>
+    <mergeCell ref="A2:A17"/>
+    <mergeCell ref="A19:A62"/>
+    <mergeCell ref="A64:A139"/>
+    <mergeCell ref="A141:A159"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E16 E150:E167 E137:E148 E60:E135 E18:E58" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E17 E161:E178 E141:E159 E64:E139 E19:E62" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not started, In progress, Deployed in production, Live Completed,Not Applicable "</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C50" r:id="rId1" tooltip="custrecord_sync_to_salesforce" display="javascript:void(%22help%22)" xr:uid="{96224D46-62AD-48F9-B7FB-0DA44BD7F0A7}"/>
-    <hyperlink ref="C51" r:id="rId2" tooltip="custrecord_sf_uph_internal_id" display="javascript:void(%22help%22)" xr:uid="{42105581-A6C8-48AB-AA04-1BA54304915E}"/>
-    <hyperlink ref="C52" r:id="rId3" tooltip="custrecord_usage_status" display="javascript:void(%22help%22)" xr:uid="{B2FFEC19-B90A-40B0-9A6A-9F961EDC135B}"/>
-    <hyperlink ref="C53" r:id="rId4" tooltip="custrecord_usage_internal_id" display="javascript:void(%22help%22)" xr:uid="{8DE219AC-5D93-44D0-8B2B-57705080D81E}"/>
-    <hyperlink ref="C26" r:id="rId5" tooltip="custrecordsf_subscription_status_updated" display="javascript:void(%22help%22)" xr:uid="{05F3077C-125C-41A2-8EEE-7B5A9697A380}"/>
+    <hyperlink ref="C54" r:id="rId1" tooltip="custrecord_sync_to_salesforce" display="javascript:void(%22help%22)" xr:uid="{96224D46-62AD-48F9-B7FB-0DA44BD7F0A7}"/>
+    <hyperlink ref="C55" r:id="rId2" tooltip="custrecord_sf_uph_internal_id" display="javascript:void(%22help%22)" xr:uid="{42105581-A6C8-48AB-AA04-1BA54304915E}"/>
+    <hyperlink ref="C56" r:id="rId3" tooltip="custrecord_usage_status" display="javascript:void(%22help%22)" xr:uid="{B2FFEC19-B90A-40B0-9A6A-9F961EDC135B}"/>
+    <hyperlink ref="C57" r:id="rId4" tooltip="custrecord_usage_internal_id" display="javascript:void(%22help%22)" xr:uid="{8DE219AC-5D93-44D0-8B2B-57705080D81E}"/>
+    <hyperlink ref="C30" r:id="rId5" tooltip="custrecordsf_subscription_status_updated" display="javascript:void(%22help%22)" xr:uid="{05F3077C-125C-41A2-8EEE-7B5A9697A380}"/>
+    <hyperlink ref="C32" r:id="rId6" tooltip="custrecord_subscription_attached" display="javascript:void(%22help%22)" xr:uid="{346B1875-F9DE-4EFA-A194-B53AA3844608}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>